<commit_message>
Apply dual coil Z positioning design
</commit_message>
<xml_diff>
--- a/docs/PTC_Mask_Transfer_4Axis_Design_Draft.xlsx
+++ b/docs/PTC_Mask_Transfer_4Axis_Design_Draft.xlsx
@@ -34,6 +34,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24_HMI_4軸畫面" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25_4軸CODEX封口清單" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26_IO不可新增與待確認" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_IO補充_雙線圈版" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27_雙線圈控制標準" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -2716,16 +2718,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="56" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2756,6 +2758,11 @@
       </c>
       <c r="F1" s="14" t="inlineStr">
         <is>
+          <t>互鎖/安全</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
           <t>備註</t>
         </is>
       </c>
@@ -2788,7 +2795,12 @@
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
-          <t>Auto只允許Axis1/2/3；Axis4不參與</t>
+          <t>Axis4 Auto禁止</t>
+        </is>
+      </c>
+      <c r="G2" s="16" t="inlineStr">
+        <is>
+          <t>Auto只允許Axis1/2/3</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2817,7 @@
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
-          <t>Y0011 ON、Y0012 OFF</t>
+          <t>Y0011 ON；Y0012 OFF</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
@@ -2815,12 +2827,17 @@
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>Timeout K310</t>
+          <t>K310</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
-          <t>使用既有正式點位，不新增Y0025/X0044</t>
+          <t>Y0011/Y0012互斥</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>左右2支伸出磁簧串聯後才完成</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2854,7 @@
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Y0013 ON、Y0014 OFF</t>
+          <t>Y0013 ON；Y0014 OFF</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
@@ -2847,12 +2864,17 @@
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>Timeout K311</t>
+          <t>K311</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>使用既有正式點位，不新增Y0026/X0046</t>
+          <t>Y0013/Y0014互斥</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>前後2支伸出磁簧串聯後才完成</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2901,17 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>K312 光罩不在席</t>
+          <t>K312</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>Z升起前必要條件</t>
+          <t>若X0026 OFF禁止Z上升</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Z升降前必要條件</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2933,7 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>M4551 ON + Busy OFF + 誤差&lt;=D4504</t>
+          <t>M4551 ON + M4527 Busy OFF + M4518 Alarm OFF + 誤差&lt;=D4504</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
@@ -2916,7 +2943,12 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>平台位高度現場實測</t>
+          <t>啟動前再確認X0016+X0020+X0026+M4517</t>
+        </is>
+      </c>
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>平台位高度現場Teach</t>
         </is>
       </c>
     </row>
@@ -2933,12 +2965,12 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Y0011 OFF、Y0012 ON、Y0013 OFF、Y0014 ON</t>
+          <t>Y0011 OFF；Y0012 ON；Y0013 OFF；Y0014 ON</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>X0017 ON 且 X0021 ON</t>
+          <t>X0017 AND X0021</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
@@ -2948,7 +2980,12 @@
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>定位縮回後才可進Barcode高度</t>
+          <t>Y0011/Y0012不可同時ON；Y0013/Y0014不可同時ON</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>未全部縮回不可進Barcode位</t>
         </is>
       </c>
     </row>
@@ -2970,7 +3007,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>M4552 ON + Busy OFF + 誤差&lt;=D4504</t>
+          <t>M4552 ON + M4527 Busy OFF + M4518 Alarm OFF + 誤差&lt;=D4504</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
@@ -2980,7 +3017,12 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Barcode高度現場實測</t>
+          <t>定位縮回完成才允許</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>Barcode高度現場Teach</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3054,12 @@
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>KEYENCE SR-2000W；通訊格式需實測</t>
+          <t>通訊Timeout需停在S389</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Barcode型號依BOM/採購版統一；若目前BOM為SR-1000W，文件先以SR-1000W</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3076,7 @@
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>PLC/HMI比對D6300~D6349與D6350~D6399</t>
+          <t>比較Storage Barcode與Mask Barcode</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -3044,7 +3091,12 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>Barcode OFF 記錄BYPASS</t>
+          <t>NG不得直接PASS</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>Barcode OFF記錄BYPASS</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3128,12 @@
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>HMI彈窗，不需要操作紀錄</t>
+          <t>Popup Hold</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>NG返回來源盒</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3145,7 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>Z升降回安全/原點等待位</t>
+          <t>Z升降回Home</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
@@ -3098,7 +3155,7 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>M4550或M4553 ON + Busy OFF</t>
+          <t>M4550 Home Complete + M4527 Busy OFF + M4518 Alarm OFF</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
@@ -3108,7 +3165,12 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>完成後通知X回檢查位</t>
+          <t>固定回Home，不用M4553替代</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>需求若改安全等待位再另定</t>
         </is>
       </c>
     </row>
@@ -3133,8 +3195,17 @@
           <t>主流程收到M6103</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr"/>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>X軸才可回Inspection</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>M6103=Z/Barcode流程完成且Z升降在安全位</t>
         </is>
@@ -3158,7 +3229,7 @@
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>X軸完成回放</t>
+          <t>X軸回放完成</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
@@ -3168,7 +3239,12 @@
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>不得自動轉Axis4</t>
+          <t>Axis4不動作</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>Barcode/Visual NG共同回收</t>
         </is>
       </c>
     </row>
@@ -3193,8 +3269,17 @@
           <t>HMI排除後回初始化/安全位</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr"/>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>所有定位閥不可同時ON</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>停機或警告依Alarm表</t>
         </is>
@@ -6476,7 +6561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6960,6 +7045,210 @@
           <t>依業主標準決定等級。</t>
         </is>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Z定位雙線圈互鎖異常</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>停機</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Y0011/Y0012或Y0013/Y0014同時ON</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>立即RST同組輸出並Alarm</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>K360</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>需檢查PLC程式/HMI手動按鈕互鎖</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="n"/>
+      <c r="H13" s="16" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Z定位伸出Timeout</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>停機</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>S301/S302未於時間內達X0016/X0020</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>停止Z流程，保持/切除依氣路策略</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>K310/K311</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>檢查氣壓、磁簧、閥線圈</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="n"/>
+      <c r="H14" s="16" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Z定位縮回Timeout</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>停機</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>S305未於時間內達X0017 AND X0021</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>禁止Z移到Barcode位</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>K321</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>檢查機構干涉與閥線圈</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="16" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Z定位雙線圈互鎖異常</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>停機</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Y0011/Y0012或Y0013/Y0014同時ON</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>立即RST同組輸出並Alarm</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>K360</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>需檢查PLC程式/HMI手動按鈕互鎖</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="16" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Z定位伸出Timeout</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>停機</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>S301/S302未於時間內達X0016/X0020</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>停止Z流程，保持/切除依氣路策略</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>K310/K311</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>檢查氣壓、磁簧、閥線圈</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="n"/>
+      <c r="H17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Z定位縮回Timeout</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>停機</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>S305未於時間內達X0017 AND X0021</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>禁止Z移到Barcode位</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>K321</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>檢查機構干涉與閥線圈</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="16" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8626,47 +8915,47 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Seq</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B1" s="14" t="inlineStr">
         <is>
-          <t>流程</t>
+          <t>流程段</t>
         </is>
       </c>
       <c r="C1" s="14" t="inlineStr">
         <is>
-          <t>動作</t>
+          <t>主要動作</t>
         </is>
       </c>
       <c r="D1" s="14" t="inlineStr">
         <is>
-          <t>條件/回授</t>
+          <t>使用軸/輸出</t>
         </is>
       </c>
       <c r="E1" s="14" t="inlineStr">
         <is>
-          <t>異常</t>
+          <t>完成條件</t>
         </is>
       </c>
       <c r="F1" s="14" t="inlineStr">
         <is>
-          <t>M/D/IO</t>
+          <t>異常處理</t>
         </is>
       </c>
       <c r="G1" s="14" t="inlineStr">
@@ -8686,27 +8975,27 @@
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>Safety/Air/FFU/Init/Axis Ready/Material State/功能Enable檢查。</t>
+          <t>確認Safety/Air/FFU/初始化/Barcode條件</t>
         </is>
       </c>
       <c r="D2" s="16" t="inlineStr">
         <is>
-          <t>Barcode Enable ON時M6301必須ON。</t>
+          <t>X0000/X0001/X0036/X0037/M1125/M1225/M1425</t>
         </is>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
-          <t>任一不成立禁止Start</t>
+          <t>Ready成立</t>
         </is>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
-          <t>X0000/X0001/M6300/M6301</t>
+          <t>不成立禁止啟動</t>
         </is>
       </c>
       <c r="G2" s="16" t="inlineStr">
         <is>
-          <t>Safety/Air/FFU不可Bypass。</t>
+          <t>Barcode Enable ON時需Storage Barcode Valid</t>
         </is>
       </c>
     </row>
@@ -8716,32 +9005,32 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>X取來源</t>
+          <t>X取來源盒</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
-          <t>X橫移到來源，X升降下降，夾爪Close，真空ON。</t>
+          <t>X橫移到來源位，X升降到取片位，夾爪關，真空ON</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>夾爪Close + Vacuum OK，真空位二次確認。</t>
+          <t>Axis1/Axis2/Y0010/Y0015</t>
         </is>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>K180/K200</t>
+          <t>X0015+X0027</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
-          <t>S100/S150/S200</t>
+          <t>真空NG-&gt;S189/S299</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>正向來源Storage；反向來源Load。</t>
+          <t>正向來源=儲存盒；反向來源=上機盒</t>
         </is>
       </c>
     </row>
@@ -8751,61 +9040,69 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>X移Inspection</t>
+          <t>X真空確認上升</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>X升降上位，X橫移到Inspection，X升降下降。</t>
+          <t>上升約10mm到真空確認位，再確認真空OK</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>X到Inspection且X升降到放/取位。</t>
+          <t>Axis2/M4330</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>K150/K160</t>
+          <t>X0027保持ON</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>M4151/M435x</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="inlineStr"/>
+          <t>真空掉落停機</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>確認後升到上位</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n">
+      <c r="A5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>放到Inspection</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>破真空，夾爪Open，光罩在席確認。</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>X0026 ON。</t>
-        </is>
-      </c>
-      <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>K201/K230</t>
-        </is>
-      </c>
-      <c r="F5" s="19" t="inlineStr">
-        <is>
-          <t>X0026/Y0016</t>
-        </is>
-      </c>
-      <c r="G5" s="19" t="inlineStr"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>X移到檢查位</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>X升降上位後，X橫移到檢查位</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Axis1</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>M4151 ON</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Axis Alarm停機</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>到位後才下降</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="n">
@@ -8813,32 +9110,32 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>X離開Clear</t>
+          <t>X放到檢查站</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>X升降上位，X橫移離開檢查干涉區。</t>
+          <t>X升降到檢查放位，破真空，夾爪開</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>X安全位到位後才SET M6100。</t>
+          <t>Axis2/Y0016/Y0007</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>K171</t>
+          <t>X0014+X0026</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>M6100</t>
+          <t>光罩未在席-&gt;Alarm</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>保護Z軸不撞。</t>
+          <t>放完X回上位再離開干涉區</t>
         </is>
       </c>
     </row>
@@ -8848,32 +9145,32 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Z定位與Barcode</t>
+          <t>X離開檢查位</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>左右定位伸出、前後定位伸出、Z到Platform、定位縮回、Z到Barcode。</t>
+          <t>X升降回上位，X橫移離開檢查區</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>X0044/X0046/X0045/X0047/M4551/M4552。</t>
+          <t>Axis1/Axis2</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>K180/K240</t>
+          <t>X已Clear</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>S300</t>
+          <t>未Clear禁止Z</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Axis3自動。</t>
+          <t>避免Z軸動作干涉</t>
         </is>
       </c>
     </row>
@@ -8883,102 +9180,102 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Barcode Compare</t>
+          <t>Z左右定位伸出</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>SR-2000W讀取Mask Barcode並比對Storage Barcode。</t>
+          <t>左右雙線圈閥伸出</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>M6304 OK；NG進Return。</t>
+          <t>Y0011 ON/Y0012 OFF</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>K181/K182</t>
+          <t>X0016 ON</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>D6300/D6350/D6400</t>
+          <t>K310</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Barcode OFF則BYPASS記錄。</t>
+          <t>2支磁簧串聯</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="n">
+      <c r="A9" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Visual確認</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>若Visual Enable ON，HMI彈窗人工OK/NG。</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>M6502 OK；M6503 NG進Return。</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>K260</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>M6500~M6504/D6500</t>
-        </is>
-      </c>
-      <c r="G9" s="18" t="inlineStr">
-        <is>
-          <t>Visual OFF則BYPASS。</t>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Z前後定位伸出</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>前後雙線圈閥伸出</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Y0013 ON/Y0014 OFF</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>X0020 ON</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>K311</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>2支磁簧串聯</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n">
+      <c r="A10" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Z回安全</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Z回Home/安全等待位。</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>M4550/M4553 ON後SET M6103。</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>K240</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>M6103</t>
-        </is>
-      </c>
-      <c r="G10" s="19" t="inlineStr">
-        <is>
-          <t>X才可進檢查位。</t>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Z升平台位</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>確認X0026後Z升到平台位</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Axis3/M4521/D4514</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>M4551 ON</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>K320</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>啟動前需X0016+X0020+X0026</t>
         </is>
       </c>
     </row>
@@ -8988,30 +9285,34 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>X取Inspection</t>
+          <t>Z定位縮回</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>X回Inspection，夾爪Close，真空ON，升降上位。</t>
+          <t>左右/前後雙線圈閥縮回</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>Vacuum OK + M4350。</t>
+          <t>Y0012 ON/Y0014 ON</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>K200/K160</t>
+          <t>X0017 AND X0021</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>S131/S163</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr"/>
+          <t>K321</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>縮回後才可去Barcode</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="n">
@@ -9019,92 +9320,104 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>PASS目的地放片</t>
+          <t>Z到Barcode位</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>正向放Load；反向放Storage。</t>
+          <t>Z升降到掃碼高度</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>放片完成。</t>
+          <t>Axis3/M4522/D4510</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>K201</t>
+          <t>M4552 ON</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>S141/S171</t>
-        </is>
-      </c>
-      <c r="G12" s="16" t="inlineStr"/>
+          <t>K322</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>高度現場Teach</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="n">
+      <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>NG Return</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>正向NG回Storage；反向NG回Load。</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Return放片完成。</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>K201</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>S380後接X Return</t>
-        </is>
-      </c>
-      <c r="G13" s="18" t="inlineStr">
-        <is>
-          <t>不得Pass到目的地。</t>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Barcode/Visual</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>掃碼、比對、目視檢查選配</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>M630x/M650x</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>OK/BYPASS</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>NG-&gt;回來源盒</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Axis4不參與Auto</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>Cycle Complete Popup</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>HMI顯示流程完成，允許開門。</t>
-        </is>
-      </c>
-      <c r="D14" s="17" t="inlineStr">
-        <is>
-          <t>M6600 ON。</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="inlineStr"/>
-      <c r="F14" s="17" t="inlineStr">
-        <is>
-          <t>M6600/M6601/Y0027</t>
-        </is>
-      </c>
-      <c r="G14" s="17" t="inlineStr"/>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Z回Home</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Z升降回Home</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Axis3/M4520/D4512</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>M4550 ON</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>K350</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>固定Home Complete</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="n">
@@ -9112,32 +9425,32 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>盒蓋關閉後破真空</t>
+          <t>X回檢查位取片</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>Storage Lid/Load Lid Closed後破真空。</t>
+          <t>X回檢查位，下降取片，真空確認，上升</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>X0052/X0053 ON。</t>
+          <t>Axis1/Axis2/Y0010/Y0015</t>
         </is>
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>K201</t>
+          <t>X0027 ON</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
-          <t>Y0030/Y0031</t>
+          <t>真空NG停機</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>兩盒獨立判斷。</t>
+          <t>準備送目的盒</t>
         </is>
       </c>
     </row>
@@ -9147,28 +9460,67 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>取出兩盒完成</t>
+          <t>X送目的盒</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>Storage Box Present OFF + Load Box Present OFF。</t>
+          <t>PASS送目的盒；NG回來源盒</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>X0022 OFF + X0024 OFF。</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr"/>
+          <t>Axis1/Axis2/Y0016/Y0007</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>放片完成</t>
+        </is>
+      </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>M6604/D6600</t>
+          <t>未到位/真空異常停機</t>
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>回Ready。</t>
+          <t>正反向依D6100/M6002/M6003</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Cycle Complete</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>允許開門/移除盒，等待兩盒移除</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>M6600/Y0020/Y0022/X0022/X0024</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>X0022 OFF AND X0024 OFF</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>逾時警告</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>不新增門鎖X/Y，門鎖若需PLC監看另走擴充點位</t>
         </is>
       </c>
     </row>
@@ -12215,15 +12567,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="74" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12234,355 +12586,385 @@
       </c>
       <c r="B1" s="14" t="inlineStr">
         <is>
-          <t>等級</t>
+          <t>優先級</t>
         </is>
       </c>
       <c r="C1" s="14" t="inlineStr">
         <is>
-          <t>項目</t>
+          <t>確認/修改事項</t>
         </is>
       </c>
       <c r="D1" s="14" t="inlineStr">
         <is>
-          <t>判定</t>
+          <t>CODEX結果</t>
         </is>
       </c>
       <c r="E1" s="14" t="inlineStr">
         <is>
-          <t>設計處理</t>
+          <t>理由/替代方案</t>
         </is>
       </c>
       <c r="F1" s="14" t="inlineStr">
         <is>
-          <t>位置</t>
+          <t>實際修改位置</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="n">
+      <c r="A2" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>2軸版升級為4軸完整定義</t>
-        </is>
-      </c>
-      <c r="D2" s="16" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>正式X/Y點位不可任意新增</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>完成</t>
         </is>
       </c>
-      <c r="E2" s="16" t="inlineStr">
-        <is>
-          <t>Axis1~4 M/D/S/HMI架構已列。</t>
-        </is>
-      </c>
-      <c r="F2" s="16" t="inlineStr">
-        <is>
-          <t>00_4軸新設計總覽</t>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>02_XY點位表只保留BOM/PLC已定義點位</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>02_XY點位表</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Auto只允許Axis1/2/3</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Z定位採4DI+4DO雙線圈版</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>完成</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
-        <is>
-          <t>Axis4明確手動限定，Auto禁止。</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>X0016/X0017/X0020/X0021 + Y0011/Y0012/Y0013/Y0014</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>01_IO補充_雙線圈版</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>廢止X0044~X0047、Y0025/Y0026舊方案</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>避免PLC/HMI/電路圖引用不同地址</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>01_IO補充_雙線圈版、26_IO不可新增與待確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>S301/S305左右雙線圈互斥</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>Y0011與Y0012不可同時ON</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>12_流程_Z升降_Barcode_S300</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>S302/S305前後雙線圈互斥</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>Y0013與Y0014不可同時ON</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>12_流程_Z升降_Barcode_S300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Auto總流程改用正式Z定位點位</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>21表使用X0016/X0020/X0017/X0021</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>21_4軸Auto完整流程</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Axis4 Z旋轉Auto禁止</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Axis4只允許工程/手動調機</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>13_流程_Z旋轉手動_S400</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>Axis3 Z升降Servo Device Map</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>Barcode型號與BOM統一</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>待確認</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>若BOM為SR-1000W，文件以SR-1000W；若採購改SR-2000W須同步BOM</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>12_S300、23_Barcode_History、BOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>S304啟動前再確認定位與光罩</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>完成</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>M4517/M4518/M452x/M455x與D451x/D455x。</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>06_M軸3_Z升降 / 08_D資料參數</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Axis4 Manual Device Map</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>X0016+X0020+X0026+Axis3 Ready</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>12_流程_Z升降_Barcode_S300</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>S310固定回Home</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>完成</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>M4717/M4718/M472x/M473x/M475x與D471x。</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>07_M軸4_Z旋轉 / 13_流程_Z旋轉手動_S400</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Z定位氣缸4DI/2DO</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>完成條件只認M4550 Home Complete，不以M4553替代</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>12_流程_Z升降_Barcode_S300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Fault Output Matrix補雙線圈故障策略</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>完成</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>X0044~X0047、Y0025~Y0026正式配置。</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>02_XY點位表 / 01_IO新增與配置</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>Z完整Sequence</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>完成</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>LR定位、FB定位、Mask Presence、Platform、縮回、Barcode、Home。</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>12_流程_Z升降_Barcode_S300</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>Barcode Enable與Storage Valid</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>完成</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>M6300/M6301與D6300起始區。</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>03_M共用_HMI_Barcode / 23_Barcode_History設計</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Visual Enable與人工判定</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>完成</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>M6500~M6504、D6500/D6502。</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>22_功能Enable矩陣 / 24_HMI_4軸畫面</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Cycle Complete與取盒</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>完成</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>M6600~M6604、X0052/X0053、Y0030/Y0031。</t>
-        </is>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>21_4軸Auto完整流程</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>異常時禁止同組雙線圈同時ON，安全/氣壓異常依停機策略處理</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>18_Fault_Output_Matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>Barcode History 1000筆</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>設計完成/實作待HMI</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>建議用HMI Ring Buffer/Data Logging，不讓PLC搬移1000筆字串。</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>23_Barcode_History設計</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>現場Release</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>仍需SR-2000W、Z高度、Tolerance、氣缸、真空、安全策略實測。</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>需實測SR通訊、Z高度、Tolerance、Safety Stop、真空/煞車策略</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>16_驗收_Release_Gate</t>
         </is>
@@ -12768,6 +13150,644 @@
       <c r="E6" s="17" t="inlineStr">
         <is>
           <t>不得新增 Y0030/Y0031</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>分類</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>正式點位</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>硬體/接線定義</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>流程使用</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>判定</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DI</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>X0016</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>左右定位伸出完成</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>左右2支氣缸伸出磁簧串聯後進PLC</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>S301完成條件</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G2" s="17" t="inlineStr">
+        <is>
+          <t>ON=兩支皆伸出</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DI</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>X0017</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>左右定位縮回完成</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>左右2支氣缸縮回磁簧串聯後進PLC</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>S305完成條件</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>ON=兩支皆縮回</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DI</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>X0020</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>前後定位伸出完成</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>前後2支氣缸伸出磁簧串聯後進PLC</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>S302完成條件</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>ON=兩支皆伸出</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DI</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>X0021</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>前後定位縮回完成</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>前後2支氣缸縮回磁簧串聯後進PLC</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>S305完成條件</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>ON=兩支皆縮回</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DO</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Y0011</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>左右定位伸出線圈</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>雙線圈閥A線圈</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>S301</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>必須與Y0012互鎖，不可同時ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DO</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Y0012</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>左右定位縮回線圈</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>雙線圈閥B線圈</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>S305</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>必須與Y0011互鎖，不可同時ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DO</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Y0013</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>前後定位伸出線圈</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>雙線圈閥A線圈</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>S302</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>必須與Y0014互鎖，不可同時ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Z定位DO</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Y0014</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>前後定位縮回線圈</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>雙線圈閥B線圈</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>S305</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>正式採用</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>必須與Y0013互鎖，不可同時ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>廢止</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>X0044~X0047</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>舊增補Z定位DI</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>非BOM/PLC正式點位</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>不得引用</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>廢止</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>正式設計不得出現在02_XY點位表</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>廢止</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Y0025/Y0026</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>舊增補Z定位DO</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>錯誤4DI/2DO方案</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>不得引用</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>廢止</t>
+        </is>
+      </c>
+      <c r="G11" s="18" t="inlineStr">
+        <is>
+          <t>正式設計不得出現在02_XY點位表</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>對象</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>伸出線圈</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>縮回線圈</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>伸出完成</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>縮回完成</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>PLC寫法原則</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>異常判定</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>檢查站左右定位</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Y0011</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Y0012</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>X0016</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>X0017</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>伸出時：Y0011=ON且Y0012=OFF；縮回時：Y0011=OFF且Y0012=ON；Y0011/Y0012不可同時ON</t>
+        </is>
+      </c>
+      <c r="G2" s="16" t="inlineStr">
+        <is>
+          <t>同時ON為程式錯誤；Timeout未到位為停機異常</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>檢查站前後定位</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Y0013</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Y0014</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>X0020</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>X0021</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>伸出時：Y0013=ON且Y0014=OFF；縮回時：Y0013=OFF且Y0014=ON；Y0013/Y0014不可同時ON</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>同時ON為程式錯誤；Timeout未到位為停機異常</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Fault/EMO/Air OFF</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>依停機策略</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>依停機策略</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>保留監看</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>保留監看</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>不得在異常中反覆切換線圈；先進Alarm等待人工排除</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>現場需確認雙線圈閥斷電是否保持最後位置</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>手動調機</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>HMI手動按鈕</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>HMI手動按鈕</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>對應DI</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>對應DI</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>工程模式才允許，且同組互鎖</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>未到位顯示Alarm/Warning</t>
         </is>
       </c>
     </row>

</xml_diff>